<commit_message>
refactor: make build rules class neutral
</commit_message>
<xml_diff>
--- a/public/designer-data/player_build.xlsx
+++ b/public/designer-data/player_build.xlsx
@@ -2372,9 +2372,6 @@
       <c r="A2" t="s">
         <v>22</v>
       </c>
-      <c r="B2" t="s">
-        <v>6</v>
-      </c>
       <c r="C2" t="s">
         <v>23</v>
       </c>
@@ -2401,9 +2398,6 @@
       <c r="A3" t="s">
         <v>27</v>
       </c>
-      <c r="B3" t="s">
-        <v>6</v>
-      </c>
       <c r="C3" t="s">
         <v>28</v>
       </c>
@@ -2430,9 +2424,6 @@
       <c r="A4" t="s">
         <v>31</v>
       </c>
-      <c r="B4" t="s">
-        <v>6</v>
-      </c>
       <c r="C4" t="s">
         <v>32</v>
       </c>
@@ -2459,9 +2450,6 @@
       <c r="A5" t="s">
         <v>35</v>
       </c>
-      <c r="B5" t="s">
-        <v>6</v>
-      </c>
       <c r="C5" t="s">
         <v>36</v>
       </c>
@@ -2488,9 +2476,6 @@
       <c r="A6" t="s">
         <v>37</v>
       </c>
-      <c r="B6" t="s">
-        <v>6</v>
-      </c>
       <c r="C6" t="s">
         <v>38</v>
       </c>
@@ -2516,9 +2501,6 @@
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>39</v>
-      </c>
-      <c r="B7" t="s">
-        <v>6</v>
       </c>
       <c r="C7" t="s">
         <v>40</v>

</xml_diff>

<commit_message>
fix: distinguish bear tank skill icons
</commit_message>
<xml_diff>
--- a/public/designer-data/player_build.xlsx
+++ b/public/designer-data/player_build.xlsx
@@ -131,10 +131,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ­ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ³ ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ°ÃÂÃÂ£ÃÂÃÂÃÂÃÂ´ÃÂÃÂ£ÃÂÃÂÃÂÃÂ·ÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂ«ÃÂÃÂ§ÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂ ÃÂÃÂªÃÂÃÂ³ÃÂÃÂ ÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂ¥ÃÂÃÂ®ÃÂÃÂÃÂÃÂ¤ÃÂÃÂ½ÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂ¦ÃÂÃÂÃÂÃÂ°ÃÂÃÂ§ÃÂÃÂ´ÃÂÃÂ°ÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂ«ÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -166,10 +166,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ­ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ³ ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ°ÃÂÃÂ£ÃÂÃÂÃÂÃÂ´ÃÂÃÂ£ÃÂÃÂÃÂÃÂ·ÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂ«ÃÂÃÂ§ÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂ ÃÂÃÂªÃÂÃÂ³ÃÂÃÂ ÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂ¥ÃÂÃÂ®ÃÂÃÂÃÂÃÂ¤ÃÂÃÂ½ÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂ¦ÃÂÃÂÃÂÃÂ°ÃÂÃÂ§ÃÂÃÂ´ÃÂÃÂ°ÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂ«ÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -10836,7 +10836,7 @@
         <v>低吼</v>
       </c>
       <c r="C51" t="str">
-        <v>bear-claw</v>
+        <v>bear-skill-growl</v>
       </c>
       <c r="D51" t="str">
         <v>skill</v>
@@ -10853,7 +10853,7 @@
         <v>裂伤</v>
       </c>
       <c r="C52" t="str">
-        <v>bear-claw</v>
+        <v>bear-skill-mangle</v>
       </c>
       <c r="D52" t="str">
         <v>skill</v>
@@ -10870,7 +10870,7 @@
         <v>痛击</v>
       </c>
       <c r="C53" t="str">
-        <v>bear-claw</v>
+        <v>bear-skill-thrash</v>
       </c>
       <c r="D53" t="str">
         <v>skill</v>
@@ -10887,7 +10887,7 @@
         <v>迎头痛击</v>
       </c>
       <c r="C54" t="str">
-        <v>bear-claw</v>
+        <v>bear-skill-skull-bash</v>
       </c>
       <c r="D54" t="str">
         <v>skill</v>
@@ -10904,7 +10904,7 @@
         <v>铁鬃</v>
       </c>
       <c r="C55" t="str">
-        <v>bear-claw</v>
+        <v>bear-skill-ironfur</v>
       </c>
       <c r="D55" t="str">
         <v>skill</v>
@@ -10921,7 +10921,7 @@
         <v>狂暴回复</v>
       </c>
       <c r="C56" t="str">
-        <v>bear-claw</v>
+        <v>bear-skill-frenzied-regeneration</v>
       </c>
       <c r="D56" t="str">
         <v>skill</v>
@@ -10938,7 +10938,7 @@
         <v>横扫</v>
       </c>
       <c r="C57" t="str">
-        <v>bear-claw</v>
+        <v>bear-skill-swipe</v>
       </c>
       <c r="D57" t="str">
         <v>skill</v>
@@ -10955,7 +10955,7 @@
         <v>月火术</v>
       </c>
       <c r="C58" t="str">
-        <v>bear-claw</v>
+        <v>bear-skill-moonfire</v>
       </c>
       <c r="D58" t="str">
         <v>skill</v>
@@ -10972,7 +10972,7 @@
         <v>树皮术</v>
       </c>
       <c r="C59" t="str">
-        <v>bear-claw</v>
+        <v>bear-skill-barkskin</v>
       </c>
       <c r="D59" t="str">
         <v>skill</v>
@@ -10989,7 +10989,7 @@
         <v>生存本能</v>
       </c>
       <c r="C60" t="str">
-        <v>bear-claw</v>
+        <v>bear-skill-survival-instincts</v>
       </c>
       <c r="D60" t="str">
         <v>skill</v>
@@ -11006,7 +11006,7 @@
         <v>明月普照</v>
       </c>
       <c r="C61" t="str">
-        <v>bear-claw</v>
+        <v>bear-skill-lunar-beam</v>
       </c>
       <c r="D61" t="str">
         <v>skill</v>
@@ -11023,7 +11023,7 @@
         <v>乌索克的化身</v>
       </c>
       <c r="C62" t="str">
-        <v>bear-claw</v>
+        <v>bear-skill-incarnation-ursoc</v>
       </c>
       <c r="D62" t="str">
         <v>skill</v>
@@ -11040,7 +11040,7 @@
         <v>沉睡者之怒</v>
       </c>
       <c r="C63" t="str">
-        <v>bear-claw</v>
+        <v>bear-skill-rage-of-the-sleeper</v>
       </c>
       <c r="D63" t="str">
         <v>skill</v>
@@ -11057,7 +11057,7 @@
         <v>愈合</v>
       </c>
       <c r="C64" t="str">
-        <v>bear-claw</v>
+        <v>bear-skill-regrowth</v>
       </c>
       <c r="D64" t="str">
         <v>skill</v>
@@ -11074,7 +11074,7 @@
         <v>狂暴</v>
       </c>
       <c r="C65" t="str">
-        <v>bear-claw</v>
+        <v>bear-skill-berserk</v>
       </c>
       <c r="D65" t="str">
         <v>skill</v>
@@ -11091,7 +11091,7 @@
         <v>咆哮</v>
       </c>
       <c r="C66" t="str">
-        <v>bear-claw</v>
+        <v>bear-skill-roar</v>
       </c>
       <c r="D66" t="str">
         <v>skill</v>
@@ -11108,7 +11108,7 @@
         <v>巨熊活力</v>
       </c>
       <c r="C67" t="str">
-        <v>bear-leaf</v>
+        <v>bear-talent-great-bear-vigor</v>
       </c>
       <c r="D67" t="str">
         <v>talent</v>
@@ -11125,7 +11125,7 @@
         <v>厚皮</v>
       </c>
       <c r="C68" t="str">
-        <v>bear-leaf</v>
+        <v>bear-talent-thick-hide</v>
       </c>
       <c r="D68" t="str">
         <v>talent</v>
@@ -11142,7 +11142,7 @@
         <v>熊威</v>
       </c>
       <c r="C69" t="str">
-        <v>bear-leaf</v>
+        <v>bear-talent-ursine-threat</v>
       </c>
       <c r="D69" t="str">
         <v>talent</v>
@@ -11159,7 +11159,7 @@
         <v>野性专注</v>
       </c>
       <c r="C70" t="str">
-        <v>bear-leaf</v>
+        <v>bear-talent-savage-focus</v>
       </c>
       <c r="D70" t="str">
         <v>talent</v>
@@ -11176,7 +11176,7 @@
         <v>疼痛豁免</v>
       </c>
       <c r="C71" t="str">
-        <v>bear-leaf</v>
+        <v>bear-talent-pain-immunity</v>
       </c>
       <c r="D71" t="str">
         <v>talent</v>
@@ -11193,7 +11193,7 @@
         <v>铁棘</v>
       </c>
       <c r="C72" t="str">
-        <v>bear-leaf</v>
+        <v>bear-talent-iron-thorns</v>
       </c>
       <c r="D72" t="str">
         <v>talent</v>
@@ -11210,7 +11210,7 @@
         <v>自然鼓舞</v>
       </c>
       <c r="C73" t="str">
-        <v>bear-leaf</v>
+        <v>bear-talent-natural-inspiration</v>
       </c>
       <c r="D73" t="str">
         <v>talent</v>
@@ -11227,7 +11227,7 @@
         <v>断法本能</v>
       </c>
       <c r="C74" t="str">
-        <v>bear-leaf</v>
+        <v>bear-talent-skull-bash-instinct</v>
       </c>
       <c r="D74" t="str">
         <v>talent</v>
@@ -11244,7 +11244,7 @@
         <v>破盾回响</v>
       </c>
       <c r="C75" t="str">
-        <v>bear-leaf</v>
+        <v>bear-talent-broken-bark</v>
       </c>
       <c r="D75" t="str">
         <v>talent</v>
@@ -11261,7 +11261,7 @@
         <v>野性印记</v>
       </c>
       <c r="C76" t="str">
-        <v>bear-leaf</v>
+        <v>bear-talent-mark-of-the-wild</v>
       </c>
       <c r="D76" t="str">
         <v>talent</v>
@@ -11278,7 +11278,7 @@
         <v>月下坚守</v>
       </c>
       <c r="C77" t="str">
-        <v>bear-leaf</v>
+        <v>bear-talent-moonlit-resolve</v>
       </c>
       <c r="D77" t="str">
         <v>talent</v>
@@ -11295,7 +11295,7 @@
         <v>树皮净化</v>
       </c>
       <c r="C78" t="str">
-        <v>bear-leaf</v>
+        <v>bear-talent-bark-dispelling</v>
       </c>
       <c r="D78" t="str">
         <v>talent</v>
@@ -11312,7 +11312,7 @@
         <v>回春羁绊</v>
       </c>
       <c r="C79" t="str">
-        <v>bear-leaf</v>
+        <v>bear-talent-regenerative-bond</v>
       </c>
       <c r="D79" t="str">
         <v>talent</v>
@@ -11329,7 +11329,7 @@
         <v>乌索克庇护</v>
       </c>
       <c r="C80" t="str">
-        <v>bear-leaf</v>
+        <v>bear-talent-ursoc-shelter</v>
       </c>
       <c r="D80" t="str">
         <v>talent</v>
@@ -11346,7 +11346,7 @@
         <v>水火不侵</v>
       </c>
       <c r="C81" t="str">
-        <v>bear-leaf</v>
+        <v>bear-talent-water-fire-immunity</v>
       </c>
       <c r="D81" t="str">
         <v>talent</v>
@@ -11363,7 +11363,7 @@
         <v>兽群愈合</v>
       </c>
       <c r="C82" t="str">
-        <v>bear-leaf</v>
+        <v>bear-talent-regrowth-of-the-pack</v>
       </c>
       <c r="D82" t="str">
         <v>talent</v>
@@ -11380,7 +11380,7 @@
         <v>林地守护者</v>
       </c>
       <c r="C83" t="str">
-        <v>bear-leaf</v>
+        <v>bear-talent-guardian-of-the-grove</v>
       </c>
       <c r="D83" t="str">
         <v>talent</v>
@@ -11397,7 +11397,7 @@
         <v>野性余震</v>
       </c>
       <c r="C84" t="str">
-        <v>bear-leaf</v>
+        <v>bear-talent-feral-aftershock</v>
       </c>
       <c r="D84" t="str">
         <v>talent</v>
@@ -11414,7 +11414,7 @@
         <v>巨熊绝境</v>
       </c>
       <c r="C85" t="str">
-        <v>bear-leaf</v>
+        <v>bear-talent-last-bear-stand</v>
       </c>
       <c r="D85" t="str">
         <v>talent</v>
@@ -11431,7 +11431,7 @@
         <v>春风吹又生</v>
       </c>
       <c r="C86" t="str">
-        <v>bear-leaf</v>
+        <v>bear-talent-spring-returns</v>
       </c>
       <c r="D86" t="str">
         <v>talent</v>
@@ -11448,7 +11448,7 @@
         <v>铁鬃</v>
       </c>
       <c r="C87" t="str">
-        <v>bear-aura</v>
+        <v>bear-status-ironfur</v>
       </c>
       <c r="D87" t="str">
         <v>status</v>
@@ -11465,7 +11465,7 @@
         <v>狂暴回复</v>
       </c>
       <c r="C88" t="str">
-        <v>bear-aura</v>
+        <v>bear-status-frenzied-regeneration</v>
       </c>
       <c r="D88" t="str">
         <v>status</v>
@@ -11482,7 +11482,7 @@
         <v>月火术</v>
       </c>
       <c r="C89" t="str">
-        <v>bear-aura</v>
+        <v>bear-status-moonfire</v>
       </c>
       <c r="D89" t="str">
         <v>status</v>
@@ -11499,7 +11499,7 @@
         <v>树皮术</v>
       </c>
       <c r="C90" t="str">
-        <v>bear-aura</v>
+        <v>bear-status-barkskin</v>
       </c>
       <c r="D90" t="str">
         <v>status</v>
@@ -11516,7 +11516,7 @@
         <v>生存本能</v>
       </c>
       <c r="C91" t="str">
-        <v>bear-aura</v>
+        <v>bear-status-survival-instincts</v>
       </c>
       <c r="D91" t="str">
         <v>status</v>
@@ -11533,7 +11533,7 @@
         <v>明月普照</v>
       </c>
       <c r="C92" t="str">
-        <v>bear-aura</v>
+        <v>bear-status-lunar-beam</v>
       </c>
       <c r="D92" t="str">
         <v>status</v>
@@ -11550,7 +11550,7 @@
         <v>乌索克的化身</v>
       </c>
       <c r="C93" t="str">
-        <v>bear-aura</v>
+        <v>bear-status-incarnation-ursoc</v>
       </c>
       <c r="D93" t="str">
         <v>status</v>
@@ -11567,7 +11567,7 @@
         <v>沉睡者之怒</v>
       </c>
       <c r="C94" t="str">
-        <v>bear-aura</v>
+        <v>bear-status-rage-of-the-sleeper</v>
       </c>
       <c r="D94" t="str">
         <v>status</v>
@@ -11584,7 +11584,7 @@
         <v>愈合</v>
       </c>
       <c r="C95" t="str">
-        <v>bear-aura</v>
+        <v>bear-status-regrowth</v>
       </c>
       <c r="D95" t="str">
         <v>status</v>
@@ -11635,7 +11635,7 @@
         <v>月下坚守</v>
       </c>
       <c r="C98" t="str">
-        <v>bear-aura</v>
+        <v>bear-status-moonlit-resolve</v>
       </c>
       <c r="D98" t="str">
         <v>status</v>
@@ -11652,7 +11652,7 @@
         <v>乌索克庇护</v>
       </c>
       <c r="C99" t="str">
-        <v>bear-aura</v>
+        <v>bear-status-ursoc-shelter</v>
       </c>
       <c r="D99" t="str">
         <v>status</v>
@@ -11669,7 +11669,7 @@
         <v>野性复原</v>
       </c>
       <c r="C100" t="str">
-        <v>bear-aura</v>
+        <v>bear-status-wild-recovery</v>
       </c>
       <c r="D100" t="str">
         <v>status</v>
@@ -11686,7 +11686,7 @@
         <v>野性余震</v>
       </c>
       <c r="C101" t="str">
-        <v>bear-aura</v>
+        <v>bear-status-feral-aftershock</v>
       </c>
       <c r="D101" t="str">
         <v>status</v>
@@ -11703,7 +11703,7 @@
         <v>林地守护者</v>
       </c>
       <c r="C102" t="str">
-        <v>bear-aura</v>
+        <v>bear-status-guardian-of-the-grove</v>
       </c>
       <c r="D102" t="str">
         <v>status</v>
@@ -11720,7 +11720,7 @@
         <v>痛苦之怒</v>
       </c>
       <c r="C103" t="str">
-        <v>bear-pain-rage</v>
+        <v>bear-talent-pain-rage</v>
       </c>
       <c r="D103" t="str">
         <v>talent</v>
@@ -11737,7 +11737,7 @@
         <v>怒气枯竭</v>
       </c>
       <c r="C104" t="str">
-        <v>bear-rage-lock</v>
+        <v>bear-status-rage-exhaustion</v>
       </c>
       <c r="D104" t="str">
         <v>status</v>
@@ -11754,7 +11754,7 @@
         <v>疼痛豁免护盾</v>
       </c>
       <c r="C105" t="str">
-        <v>bear-aura</v>
+        <v>bear-status-pain-immunity</v>
       </c>
       <c r="D105" t="str">
         <v>status</v>

</xml_diff>